<commit_message>
E36: guard the waste denominator with MAX(1, ...) like the other templates; rebuild samples
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Hz7DycYn6Dwb4gDvm1VWqS
</commit_message>
<xml_diff>
--- a/samples/bakery-full-5y.xlsx
+++ b/samples/bakery-full-5y.xlsx
@@ -2666,8 +2666,8 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="0"/>
-        <c:axId val="62552561"/>
-        <c:axId val="42081338"/>
+        <c:axId val="17839765"/>
+        <c:axId val="24974461"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -2788,11 +2788,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="96328969"/>
-        <c:axId val="21422302"/>
+        <c:axId val="74675383"/>
+        <c:axId val="86514201"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="62552561"/>
+        <c:axId val="17839765"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2824,7 +2824,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="42081338"/>
+        <c:crossAx val="24974461"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2832,7 +2832,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="42081338"/>
+        <c:axId val="24974461"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2871,12 +2871,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="62552561"/>
+        <c:crossAx val="17839765"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="96328969"/>
+        <c:axId val="74675383"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2908,7 +2908,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="21422302"/>
+        <c:crossAx val="86514201"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2916,7 +2916,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="21422302"/>
+        <c:axId val="86514201"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2945,7 +2945,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="96328969"/>
+        <c:crossAx val="74675383"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3370,11 +3370,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="94629950"/>
-        <c:axId val="84084865"/>
+        <c:axId val="49307601"/>
+        <c:axId val="60955298"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="94629950"/>
+        <c:axId val="49307601"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3406,7 +3406,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="84084865"/>
+        <c:crossAx val="60955298"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3414,7 +3414,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="84084865"/>
+        <c:axId val="60955298"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3453,7 +3453,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="94629950"/>
+        <c:crossAx val="49307601"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3634,7 +3634,7 @@
                   <c:v>0.316330859442882</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.281586318034303</c:v>
+                  <c:v>0.281586318034302</c:v>
                 </c:pt>
                 <c:pt idx="4">
                   <c:v>0.255332574177591</c:v>
@@ -3727,7 +3727,7 @@
                   <c:v>0.462712266442819</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.361999900076399</c:v>
+                  <c:v>0.361999900076398</c:v>
                 </c:pt>
                 <c:pt idx="3">
                   <c:v>0.304445721457148</c:v>
@@ -3741,11 +3741,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="0"/>
-        <c:axId val="64570751"/>
-        <c:axId val="73202663"/>
+        <c:axId val="51828604"/>
+        <c:axId val="27762018"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="64570751"/>
+        <c:axId val="51828604"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3777,7 +3777,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="73202663"/>
+        <c:crossAx val="27762018"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3785,7 +3785,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="73202663"/>
+        <c:axId val="27762018"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3824,7 +3824,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="64570751"/>
+        <c:crossAx val="51828604"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4016,8 +4016,8 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="0"/>
-        <c:axId val="87149749"/>
-        <c:axId val="98573043"/>
+        <c:axId val="74484853"/>
+        <c:axId val="33994403"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -4138,11 +4138,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="74779806"/>
-        <c:axId val="54978463"/>
+        <c:axId val="20087231"/>
+        <c:axId val="75227093"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="87149749"/>
+        <c:axId val="74484853"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4174,7 +4174,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="98573043"/>
+        <c:crossAx val="33994403"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4182,7 +4182,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="98573043"/>
+        <c:axId val="33994403"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4221,12 +4221,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="87149749"/>
+        <c:crossAx val="74484853"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="74779806"/>
+        <c:axId val="20087231"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4258,7 +4258,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="54978463"/>
+        <c:crossAx val="75227093"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4266,7 +4266,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="54978463"/>
+        <c:axId val="75227093"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4295,7 +4295,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="74779806"/>
+        <c:crossAx val="20087231"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4583,8 +4583,8 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="0"/>
-        <c:axId val="99892019"/>
-        <c:axId val="61016013"/>
+        <c:axId val="25273104"/>
+        <c:axId val="40792867"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -4705,11 +4705,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="55873505"/>
-        <c:axId val="94350536"/>
+        <c:axId val="3136053"/>
+        <c:axId val="84774871"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="99892019"/>
+        <c:axId val="25273104"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4741,7 +4741,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="61016013"/>
+        <c:crossAx val="40792867"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4749,7 +4749,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="61016013"/>
+        <c:axId val="40792867"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4788,12 +4788,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="99892019"/>
+        <c:crossAx val="25273104"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="55873505"/>
+        <c:axId val="3136053"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4825,7 +4825,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="94350536"/>
+        <c:crossAx val="84774871"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4833,7 +4833,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="94350536"/>
+        <c:axId val="84774871"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4862,7 +4862,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="55873505"/>
+        <c:crossAx val="3136053"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5246,11 +5246,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="0"/>
-        <c:axId val="79532440"/>
-        <c:axId val="78128852"/>
+        <c:axId val="71356892"/>
+        <c:axId val="2009010"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="79532440"/>
+        <c:axId val="71356892"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5282,7 +5282,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="78128852"/>
+        <c:crossAx val="2009010"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5290,7 +5290,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="78128852"/>
+        <c:axId val="2009010"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5329,7 +5329,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="79532440"/>
+        <c:crossAx val="71356892"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5525,11 +5525,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="0"/>
-        <c:axId val="37973469"/>
-        <c:axId val="96888523"/>
+        <c:axId val="65243778"/>
+        <c:axId val="35827928"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="37973469"/>
+        <c:axId val="65243778"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5561,7 +5561,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="96888523"/>
+        <c:crossAx val="35827928"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5569,7 +5569,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="96888523"/>
+        <c:axId val="35827928"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5608,7 +5608,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="37973469"/>
+        <c:crossAx val="65243778"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5872,11 +5872,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="44435928"/>
-        <c:axId val="47332584"/>
+        <c:axId val="49308112"/>
+        <c:axId val="94685100"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="44435928"/>
+        <c:axId val="49308112"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5908,7 +5908,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="47332584"/>
+        <c:crossAx val="94685100"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -5916,7 +5916,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="47332584"/>
+        <c:axId val="94685100"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -5955,7 +5955,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="44435928"/>
+        <c:crossAx val="49308112"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -6189,8 +6189,8 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="0"/>
-        <c:axId val="61233540"/>
-        <c:axId val="97897133"/>
+        <c:axId val="8571800"/>
+        <c:axId val="51057367"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -6503,11 +6503,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="61233540"/>
-        <c:axId val="97897133"/>
+        <c:axId val="8571800"/>
+        <c:axId val="51057367"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="61233540"/>
+        <c:axId val="8571800"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6539,7 +6539,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="97897133"/>
+        <c:crossAx val="51057367"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -6547,7 +6547,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="97897133"/>
+        <c:axId val="51057367"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -6586,7 +6586,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="61233540"/>
+        <c:crossAx val="8571800"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -7096,8 +7096,8 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="0"/>
-        <c:axId val="36099347"/>
-        <c:axId val="34918384"/>
+        <c:axId val="51361594"/>
+        <c:axId val="60963952"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="standard"/>
@@ -7260,11 +7260,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="45582842"/>
-        <c:axId val="15167407"/>
+        <c:axId val="58621285"/>
+        <c:axId val="22384456"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="36099347"/>
+        <c:axId val="51361594"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7296,7 +7296,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="34918384"/>
+        <c:crossAx val="60963952"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -7304,7 +7304,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="34918384"/>
+        <c:axId val="60963952"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7343,12 +7343,12 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="36099347"/>
+        <c:crossAx val="51361594"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:catAx>
-        <c:axId val="45582842"/>
+        <c:axId val="58621285"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7380,7 +7380,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="15167407"/>
+        <c:crossAx val="22384456"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -7388,7 +7388,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="15167407"/>
+        <c:axId val="22384456"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -7417,7 +7417,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="45582842"/>
+        <c:crossAx val="58621285"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -7927,8 +7927,8 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="100"/>
-        <c:axId val="20171895"/>
-        <c:axId val="77295525"/>
+        <c:axId val="98116798"/>
+        <c:axId val="20577458"/>
       </c:barChart>
       <c:lineChart>
         <c:grouping val="stacked"/>
@@ -8091,11 +8091,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="1"/>
-        <c:axId val="20171895"/>
-        <c:axId val="77295525"/>
+        <c:axId val="98116798"/>
+        <c:axId val="20577458"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="20171895"/>
+        <c:axId val="98116798"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8127,7 +8127,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="77295525"/>
+        <c:crossAx val="20577458"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -8135,7 +8135,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="77295525"/>
+        <c:axId val="20577458"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8174,7 +8174,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="20171895"/>
+        <c:crossAx val="98116798"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -8602,11 +8602,11 @@
         </c:ser>
         <c:gapWidth val="60"/>
         <c:overlap val="0"/>
-        <c:axId val="85634712"/>
-        <c:axId val="19014353"/>
+        <c:axId val="42380813"/>
+        <c:axId val="29818212"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="85634712"/>
+        <c:axId val="42380813"/>
         <c:scaling>
           <c:orientation val="maxMin"/>
         </c:scaling>
@@ -8638,7 +8638,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="19014353"/>
+        <c:crossAx val="29818212"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -8646,7 +8646,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="19014353"/>
+        <c:axId val="29818212"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -8685,7 +8685,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="85634712"/>
+        <c:crossAx val="42380813"/>
         <c:crosses val="max"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -14096,243 +14096,243 @@
         <v>381</v>
       </c>
       <c r="C26" s="51" t="n">
-        <f aca="false">-C14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-C14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-1962.21805714286</v>
       </c>
       <c r="D26" s="51" t="n">
-        <f aca="false">-D14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-D14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2071.23017142857</v>
       </c>
       <c r="E26" s="51" t="n">
-        <f aca="false">-E14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-E14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2180.24228571429</v>
       </c>
       <c r="F26" s="51" t="n">
-        <f aca="false">-F14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-F14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2180.24228571429</v>
       </c>
       <c r="G26" s="51" t="n">
-        <f aca="false">-G14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-G14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2180.24228571429</v>
       </c>
       <c r="H26" s="51" t="n">
-        <f aca="false">-H14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-H14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2180.24228571429</v>
       </c>
       <c r="I26" s="51" t="n">
-        <f aca="false">-I14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-I14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2180.24228571429</v>
       </c>
       <c r="J26" s="51" t="n">
-        <f aca="false">-J14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-J14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2180.24228571429</v>
       </c>
       <c r="K26" s="51" t="n">
-        <f aca="false">-K14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-K14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2180.24228571429</v>
       </c>
       <c r="L26" s="51" t="n">
-        <f aca="false">-L14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-L14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2180.24228571429</v>
       </c>
       <c r="M26" s="51" t="n">
-        <f aca="false">-M14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-M14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2725.30285714286</v>
       </c>
       <c r="N26" s="51" t="n">
-        <f aca="false">-N14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-N14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2725.30285714286</v>
       </c>
       <c r="O26" s="51" t="n">
-        <f aca="false">-O14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-O14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2313.01904091429</v>
       </c>
       <c r="P26" s="51" t="n">
-        <f aca="false">-P14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-P14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2313.01904091429</v>
       </c>
       <c r="Q26" s="51" t="n">
-        <f aca="false">-Q14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-Q14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2313.01904091429</v>
       </c>
       <c r="R26" s="51" t="n">
-        <f aca="false">-R14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-R14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2313.01904091429</v>
       </c>
       <c r="S26" s="51" t="n">
-        <f aca="false">-S14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-S14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2313.01904091429</v>
       </c>
       <c r="T26" s="51" t="n">
-        <f aca="false">-T14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-T14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2313.01904091429</v>
       </c>
       <c r="U26" s="51" t="n">
-        <f aca="false">-U14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-U14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2313.01904091429</v>
       </c>
       <c r="V26" s="51" t="n">
-        <f aca="false">-V14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-V14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2313.01904091429</v>
       </c>
       <c r="W26" s="51" t="n">
-        <f aca="false">-W14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-W14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2313.01904091429</v>
       </c>
       <c r="X26" s="51" t="n">
-        <f aca="false">-X14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-X14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2313.01904091429</v>
       </c>
       <c r="Y26" s="51" t="n">
-        <f aca="false">-Y14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-Y14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2891.27380114286</v>
       </c>
       <c r="Z26" s="51" t="n">
-        <f aca="false">-Z14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-Z14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2891.27380114286</v>
       </c>
       <c r="AA26" s="51" t="n">
-        <f aca="false">-AA14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-AA14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2453.88190050597</v>
       </c>
       <c r="AB26" s="51" t="n">
-        <f aca="false">-AB14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-AB14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2453.88190050597</v>
       </c>
       <c r="AC26" s="51" t="n">
-        <f aca="false">-AC14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-AC14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2453.88190050597</v>
       </c>
       <c r="AD26" s="51" t="n">
-        <f aca="false">-AD14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-AD14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2453.88190050597</v>
       </c>
       <c r="AE26" s="51" t="n">
-        <f aca="false">-AE14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-AE14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2453.88190050597</v>
       </c>
       <c r="AF26" s="51" t="n">
-        <f aca="false">-AF14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-AF14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2453.88190050597</v>
       </c>
       <c r="AG26" s="51" t="n">
-        <f aca="false">-AG14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-AG14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2453.88190050597</v>
       </c>
       <c r="AH26" s="51" t="n">
-        <f aca="false">-AH14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-AH14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2453.88190050597</v>
       </c>
       <c r="AI26" s="51" t="n">
-        <f aca="false">-AI14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-AI14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2453.88190050597</v>
       </c>
       <c r="AJ26" s="51" t="n">
-        <f aca="false">-AJ14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-AJ14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2453.88190050597</v>
       </c>
       <c r="AK26" s="51" t="n">
-        <f aca="false">-AK14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-AK14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-3067.35237563246</v>
       </c>
       <c r="AL26" s="51" t="n">
-        <f aca="false">-AL14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-AL14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-3067.35237563246</v>
       </c>
       <c r="AM26" s="51" t="n">
-        <f aca="false">-AM14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-AM14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2603.32330824678</v>
       </c>
       <c r="AN26" s="51" t="n">
-        <f aca="false">-AN14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-AN14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2603.32330824678</v>
       </c>
       <c r="AO26" s="51" t="n">
-        <f aca="false">-AO14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-AO14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2603.32330824678</v>
       </c>
       <c r="AP26" s="51" t="n">
-        <f aca="false">-AP14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-AP14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2603.32330824678</v>
       </c>
       <c r="AQ26" s="51" t="n">
-        <f aca="false">-AQ14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-AQ14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2603.32330824678</v>
       </c>
       <c r="AR26" s="51" t="n">
-        <f aca="false">-AR14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-AR14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2603.32330824678</v>
       </c>
       <c r="AS26" s="51" t="n">
-        <f aca="false">-AS14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-AS14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2603.32330824678</v>
       </c>
       <c r="AT26" s="51" t="n">
-        <f aca="false">-AT14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-AT14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2603.32330824678</v>
       </c>
       <c r="AU26" s="51" t="n">
-        <f aca="false">-AU14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-AU14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2603.32330824678</v>
       </c>
       <c r="AV26" s="51" t="n">
-        <f aca="false">-AV14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-AV14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2603.32330824678</v>
       </c>
       <c r="AW26" s="51" t="n">
-        <f aca="false">-AW14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
-        <v>-3254.15413530847</v>
+        <f aca="false">-AW14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
+        <v>-3254.15413530848</v>
       </c>
       <c r="AX26" s="51" t="n">
-        <f aca="false">-AX14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
-        <v>-3254.15413530847</v>
+        <f aca="false">-AX14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
+        <v>-3254.15413530848</v>
       </c>
       <c r="AY26" s="51" t="n">
-        <f aca="false">-AY14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-AY14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2761.86569771901</v>
       </c>
       <c r="AZ26" s="51" t="n">
-        <f aca="false">-AZ14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-AZ14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2761.86569771901</v>
       </c>
       <c r="BA26" s="51" t="n">
-        <f aca="false">-BA14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-BA14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2761.86569771901</v>
       </c>
       <c r="BB26" s="51" t="n">
-        <f aca="false">-BB14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-BB14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2761.86569771901</v>
       </c>
       <c r="BC26" s="51" t="n">
-        <f aca="false">-BC14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-BC14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2761.86569771901</v>
       </c>
       <c r="BD26" s="51" t="n">
-        <f aca="false">-BD14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-BD14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2761.86569771901</v>
       </c>
       <c r="BE26" s="51" t="n">
-        <f aca="false">-BE14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-BE14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2761.86569771901</v>
       </c>
       <c r="BF26" s="51" t="n">
-        <f aca="false">-BF14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-BF14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2761.86569771901</v>
       </c>
       <c r="BG26" s="51" t="n">
-        <f aca="false">-BG14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-BG14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2761.86569771901</v>
       </c>
       <c r="BH26" s="51" t="n">
-        <f aca="false">-BH14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-BH14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-2761.86569771901</v>
       </c>
       <c r="BI26" s="51" t="n">
-        <f aca="false">-BI14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-BI14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-3452.33212214876</v>
       </c>
       <c r="BJ26" s="51" t="n">
-        <f aca="false">-BJ14*Inputs!$E$24*Inputs!$E$26/MAX(0.01,1-Inputs!$E$26)</f>
+        <f aca="false">-BJ14*Inputs!$E$24*Inputs!$E$26*100/MAX(1,100-100*Inputs!$E$26)</f>
         <v>-3452.33212214876</v>
       </c>
     </row>
@@ -17623,11 +17623,11 @@
       </c>
       <c r="Q44" s="58" t="n">
         <f aca="false">Q41+Q55</f>
-        <v>12341.9074613638</v>
+        <v>12341.9074613639</v>
       </c>
       <c r="R44" s="58" t="n">
         <f aca="false">R41+R55</f>
-        <v>12328.0185724749</v>
+        <v>12328.018572475</v>
       </c>
       <c r="S44" s="58" t="n">
         <f aca="false">S41+S55</f>
@@ -18125,7 +18125,7 @@
       </c>
       <c r="T46" s="52" t="n">
         <f aca="false">T44+T45</f>
-        <v>11889.4074613638</v>
+        <v>11889.4074613639</v>
       </c>
       <c r="U46" s="52" t="n">
         <f aca="false">U44+U45</f>
@@ -18133,7 +18133,7 @@
       </c>
       <c r="V46" s="52" t="n">
         <f aca="false">V44+V45</f>
-        <v>11880.5185724749</v>
+        <v>11880.518572475</v>
       </c>
       <c r="W46" s="52" t="n">
         <f aca="false">W44+W45</f>
@@ -18430,7 +18430,7 @@
       </c>
       <c r="AI47" s="51" t="n">
         <f aca="false">AH47+AI46</f>
-        <v>436317.984699272</v>
+        <v>436317.984699273</v>
       </c>
       <c r="AJ47" s="51" t="n">
         <f aca="false">AI47+AJ46</f>
@@ -18450,7 +18450,7 @@
       </c>
       <c r="AN47" s="51" t="n">
         <f aca="false">AM47+AN46</f>
-        <v>552259.93101582</v>
+        <v>552259.931015821</v>
       </c>
       <c r="AO47" s="51" t="n">
         <f aca="false">AN47+AO46</f>
@@ -18486,7 +18486,7 @@
       </c>
       <c r="AW47" s="51" t="n">
         <f aca="false">AV47+AW46</f>
-        <v>737302.163324327</v>
+        <v>737302.163324328</v>
       </c>
       <c r="AX47" s="51" t="n">
         <f aca="false">AW47+AX46</f>
@@ -18502,11 +18502,11 @@
       </c>
       <c r="BA47" s="51" t="n">
         <f aca="false">AZ47+BA46</f>
-        <v>841707.17234765</v>
+        <v>841707.172347651</v>
       </c>
       <c r="BB47" s="51" t="n">
         <f aca="false">BA47+BB46</f>
-        <v>864346.682502251</v>
+        <v>864346.682502252</v>
       </c>
       <c r="BC47" s="51" t="n">
         <f aca="false">BB47+BC46</f>
@@ -18675,7 +18675,7 @@
       </c>
       <c r="AI48" s="51" t="n">
         <f aca="false">MAX(AH48,AI47)</f>
-        <v>436317.984699272</v>
+        <v>436317.984699273</v>
       </c>
       <c r="AJ48" s="51" t="n">
         <f aca="false">MAX(AI48,AJ47)</f>
@@ -18695,7 +18695,7 @@
       </c>
       <c r="AN48" s="51" t="n">
         <f aca="false">MAX(AM48,AN47)</f>
-        <v>552259.93101582</v>
+        <v>552259.931015821</v>
       </c>
       <c r="AO48" s="51" t="n">
         <f aca="false">MAX(AN48,AO47)</f>
@@ -18731,7 +18731,7 @@
       </c>
       <c r="AW48" s="51" t="n">
         <f aca="false">MAX(AV48,AW47)</f>
-        <v>737302.163324327</v>
+        <v>737302.163324328</v>
       </c>
       <c r="AX48" s="51" t="n">
         <f aca="false">MAX(AW48,AX47)</f>
@@ -18747,11 +18747,11 @@
       </c>
       <c r="BA48" s="51" t="n">
         <f aca="false">MAX(AZ48,BA47)</f>
-        <v>841707.17234765</v>
+        <v>841707.172347651</v>
       </c>
       <c r="BB48" s="51" t="n">
         <f aca="false">MAX(BA48,BB47)</f>
-        <v>864346.682502251</v>
+        <v>864346.682502252</v>
       </c>
       <c r="BC48" s="51" t="n">
         <f aca="false">MAX(BB48,BC47)</f>
@@ -18848,7 +18848,7 @@
       </c>
       <c r="Q49" s="51" t="n">
         <f aca="false">-(Q48-P48)*Inputs!$E$70</f>
-        <v>-2499.5755668864</v>
+        <v>-2499.57556688641</v>
       </c>
       <c r="R49" s="51" t="n">
         <f aca="false">-(R48-Q48)*Inputs!$E$70</f>
@@ -18860,11 +18860,11 @@
       </c>
       <c r="T49" s="51" t="n">
         <f aca="false">-(T48-S48)*Inputs!$E$70</f>
-        <v>-2496.7755668864</v>
+        <v>-2496.77556688641</v>
       </c>
       <c r="U49" s="51" t="n">
         <f aca="false">-(U48-T48)*Inputs!$E$70</f>
-        <v>-2495.84223355307</v>
+        <v>-2495.84223355308</v>
       </c>
       <c r="V49" s="51" t="n">
         <f aca="false">-(V48-U48)*Inputs!$E$70</f>
@@ -19028,7 +19028,7 @@
       </c>
       <c r="BJ49" s="51" t="n">
         <f aca="false">-(BJ48-BI48)*Inputs!$E$70</f>
-        <v>-8737.42911484853</v>
+        <v>-8737.42911484855</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -19085,7 +19085,7 @@
       </c>
       <c r="O50" s="52" t="n">
         <f aca="false">O46+O49</f>
-        <v>9410.18745003298</v>
+        <v>9410.187450033</v>
       </c>
       <c r="P50" s="52" t="n">
         <f aca="false">P46+P49</f>
@@ -19097,31 +19097,31 @@
       </c>
       <c r="R50" s="52" t="n">
         <f aca="false">R46+R49</f>
-        <v>9399.65411669965</v>
+        <v>9399.65411669967</v>
       </c>
       <c r="S50" s="52" t="n">
         <f aca="false">S46+S49</f>
-        <v>9396.14300558854</v>
+        <v>9396.14300558855</v>
       </c>
       <c r="T50" s="52" t="n">
         <f aca="false">T46+T49</f>
-        <v>9392.63189447743</v>
+        <v>9392.63189447744</v>
       </c>
       <c r="U50" s="52" t="n">
         <f aca="false">U46+U49</f>
-        <v>9389.12078336632</v>
+        <v>9389.12078336633</v>
       </c>
       <c r="V50" s="52" t="n">
         <f aca="false">V46+V49</f>
-        <v>9385.60967225521</v>
+        <v>9385.60967225522</v>
       </c>
       <c r="W50" s="52" t="n">
         <f aca="false">W46+W49</f>
-        <v>9382.09856114409</v>
+        <v>9382.09856114411</v>
       </c>
       <c r="X50" s="52" t="n">
         <f aca="false">X46+X49</f>
-        <v>9378.58745003298</v>
+        <v>9378.587450033</v>
       </c>
       <c r="Y50" s="52" t="n">
         <f aca="false">Y46+Y49</f>
@@ -19273,7 +19273,7 @@
       </c>
       <c r="BJ50" s="52" t="n">
         <f aca="false">BJ46+BJ49</f>
-        <v>32869.3761939541</v>
+        <v>32869.376193954</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -22575,7 +22575,7 @@
       </c>
       <c r="O70" s="51" t="n">
         <f aca="false">N67-O67</f>
-        <v>308.982288822856</v>
+        <v>308.982288822857</v>
       </c>
       <c r="P70" s="51" t="n">
         <f aca="false">O67-P67</f>
@@ -22615,7 +22615,7 @@
       </c>
       <c r="Y70" s="51" t="n">
         <f aca="false">X67-Y67</f>
-        <v>-727.771095222857</v>
+        <v>-727.771095222858</v>
       </c>
       <c r="Z70" s="51" t="n">
         <f aca="false">Y67-Z67</f>
@@ -23121,7 +23121,7 @@
       </c>
       <c r="X74" s="58" t="n">
         <f aca="false">X50-X55+X69+X70+X71</f>
-        <v>10588.9049103504</v>
+        <v>10588.9049103505</v>
       </c>
       <c r="Y74" s="58" t="n">
         <f aca="false">Y50-Y55+Y69+Y70+Y71</f>
@@ -24065,7 +24065,7 @@
       </c>
       <c r="O78" s="52" t="n">
         <f aca="false">O74+O75+O77</f>
-        <v>9161.59557823615</v>
+        <v>9161.59557823617</v>
       </c>
       <c r="P78" s="52" t="n">
         <f aca="false">P74+P75+P77</f>
@@ -24073,19 +24073,19 @@
       </c>
       <c r="Q78" s="52" t="n">
         <f aca="false">Q74+Q75+Q77</f>
-        <v>8016.260465906</v>
+        <v>8016.26046590601</v>
       </c>
       <c r="R78" s="52" t="n">
         <f aca="false">R74+R75+R77</f>
-        <v>8026.63824368378</v>
+        <v>8026.63824368379</v>
       </c>
       <c r="S78" s="52" t="n">
         <f aca="false">S74+S75+S77</f>
-        <v>8037.01602146156</v>
+        <v>8037.01602146157</v>
       </c>
       <c r="T78" s="52" t="n">
         <f aca="false">T74+T75+T77</f>
-        <v>8047.39379923934</v>
+        <v>8047.39379923935</v>
       </c>
       <c r="U78" s="52" t="n">
         <f aca="false">U74+U75+U77</f>
@@ -24093,15 +24093,15 @@
       </c>
       <c r="V78" s="52" t="n">
         <f aca="false">V74+V75+V77</f>
-        <v>8068.14935479489</v>
+        <v>8068.14935479491</v>
       </c>
       <c r="W78" s="52" t="n">
         <f aca="false">W74+W75+W77</f>
-        <v>8078.52713257267</v>
+        <v>8078.52713257268</v>
       </c>
       <c r="X78" s="52" t="n">
         <f aca="false">X74+X75+X77</f>
-        <v>8088.90491035044</v>
+        <v>8088.90491035046</v>
       </c>
       <c r="Y78" s="52" t="n">
         <f aca="false">Y74+Y75+Y77</f>
@@ -24374,7 +24374,7 @@
       </c>
       <c r="AE79" s="51" t="n">
         <f aca="false">AD80</f>
-        <v>301399.202882855</v>
+        <v>301399.202882856</v>
       </c>
       <c r="AF79" s="51" t="n">
         <f aca="false">AE80</f>
@@ -24430,7 +24430,7 @@
       </c>
       <c r="AS79" s="51" t="n">
         <f aca="false">AR80</f>
-        <v>494662.548347196</v>
+        <v>494662.548347197</v>
       </c>
       <c r="AT79" s="51" t="n">
         <f aca="false">AS80</f>
@@ -24462,7 +24462,7 @@
       </c>
       <c r="BA79" s="51" t="n">
         <f aca="false">AZ80</f>
-        <v>638115.897747846</v>
+        <v>638115.897747847</v>
       </c>
       <c r="BB79" s="51" t="n">
         <f aca="false">BA80</f>
@@ -24615,7 +24615,7 @@
       </c>
       <c r="AD80" s="52" t="n">
         <f aca="false">AD79+AD78</f>
-        <v>301399.202882855</v>
+        <v>301399.202882856</v>
       </c>
       <c r="AE80" s="52" t="n">
         <f aca="false">AE79+AE78</f>
@@ -24671,7 +24671,7 @@
       </c>
       <c r="AR80" s="52" t="n">
         <f aca="false">AR79+AR78</f>
-        <v>494662.548347196</v>
+        <v>494662.548347197</v>
       </c>
       <c r="AS80" s="52" t="n">
         <f aca="false">AS79+AS78</f>
@@ -24703,7 +24703,7 @@
       </c>
       <c r="AZ80" s="52" t="n">
         <f aca="false">AZ79+AZ78</f>
-        <v>638115.897747846</v>
+        <v>638115.897747847</v>
       </c>
       <c r="BA80" s="52" t="n">
         <f aca="false">BA79+BA78</f>
@@ -25314,39 +25314,39 @@
       </c>
       <c r="P85" s="51" t="n">
         <f aca="false">P74+P75</f>
-        <v>9339.21602146156</v>
+        <v>9339.21602146157</v>
       </c>
       <c r="Q85" s="51" t="n">
         <f aca="false">Q74+Q75</f>
-        <v>9349.59379923934</v>
+        <v>9349.59379923935</v>
       </c>
       <c r="R85" s="51" t="n">
         <f aca="false">R74+R75</f>
-        <v>9359.97157701711</v>
+        <v>9359.97157701713</v>
       </c>
       <c r="S85" s="51" t="n">
         <f aca="false">S74+S75</f>
-        <v>9370.34935479489</v>
+        <v>9370.3493547949</v>
       </c>
       <c r="T85" s="51" t="n">
         <f aca="false">T74+T75</f>
-        <v>9380.72713257267</v>
+        <v>9380.72713257268</v>
       </c>
       <c r="U85" s="51" t="n">
         <f aca="false">U74+U75</f>
-        <v>9391.10491035045</v>
+        <v>9391.10491035046</v>
       </c>
       <c r="V85" s="51" t="n">
         <f aca="false">V74+V75</f>
-        <v>9401.48268812822</v>
+        <v>9401.48268812824</v>
       </c>
       <c r="W85" s="51" t="n">
         <f aca="false">W74+W75</f>
-        <v>9411.860465906</v>
+        <v>9411.86046590602</v>
       </c>
       <c r="X85" s="51" t="n">
         <f aca="false">X74+X75</f>
-        <v>9422.23824368378</v>
+        <v>9422.23824368379</v>
       </c>
       <c r="Y85" s="51" t="n">
         <f aca="false">Y74+Y75</f>
@@ -25559,7 +25559,7 @@
       </c>
       <c r="P86" s="51" t="n">
         <f aca="false">O86+P85</f>
-        <v>31198.1019696533</v>
+        <v>31198.1019696534</v>
       </c>
       <c r="Q86" s="51" t="n">
         <f aca="false">P86+Q85</f>
@@ -25579,15 +25579,15 @@
       </c>
       <c r="U86" s="51" t="n">
         <f aca="false">T86+U85</f>
-        <v>78049.8487436278</v>
+        <v>78049.8487436279</v>
       </c>
       <c r="V86" s="51" t="n">
         <f aca="false">U86+V85</f>
-        <v>87451.331431756</v>
+        <v>87451.3314317561</v>
       </c>
       <c r="W86" s="51" t="n">
         <f aca="false">V86+W85</f>
-        <v>96863.191897662</v>
+        <v>96863.1918976621</v>
       </c>
       <c r="X86" s="51" t="n">
         <f aca="false">W86+X85</f>
@@ -25595,7 +25595,7 @@
       </c>
       <c r="Y86" s="51" t="n">
         <f aca="false">X86+Y85</f>
-        <v>126245.039325131</v>
+        <v>126245.039325132</v>
       </c>
       <c r="Z86" s="51" t="n">
         <f aca="false">Y86+Z85</f>
@@ -25607,7 +25607,7 @@
       </c>
       <c r="AB86" s="51" t="n">
         <f aca="false">AA86+AB85</f>
-        <v>173414.12805599</v>
+        <v>173414.128055991</v>
       </c>
       <c r="AC86" s="51" t="n">
         <f aca="false">AB86+AC85</f>
@@ -25619,7 +25619,7 @@
       </c>
       <c r="AE86" s="51" t="n">
         <f aca="false">AD86+AE85</f>
-        <v>209407.306962954</v>
+        <v>209407.306962955</v>
       </c>
       <c r="AF86" s="51" t="n">
         <f aca="false">AE86+AF85</f>
@@ -25679,7 +25679,7 @@
       </c>
       <c r="AT86" s="51" t="n">
         <f aca="false">AS86+AT85</f>
-        <v>439350.866855478</v>
+        <v>439350.866855479</v>
       </c>
       <c r="AU86" s="51" t="n">
         <f aca="false">AT86+AU85</f>
@@ -25711,7 +25711,7 @@
       </c>
       <c r="BB86" s="51" t="n">
         <f aca="false">BA86+BB85</f>
-        <v>600129.914268306</v>
+        <v>600129.914268307</v>
       </c>
       <c r="BC86" s="51" t="n">
         <f aca="false">BB86+BC85</f>
@@ -25743,7 +25743,7 @@
       </c>
       <c r="BJ86" s="51" t="n">
         <f aca="false">BI86+BJ85</f>
-        <v>774849.79054965</v>
+        <v>774849.790549651</v>
       </c>
     </row>
     <row r="87" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -26302,11 +26302,11 @@
       </c>
       <c r="R89" s="51" t="n">
         <f aca="false">R74-R45*(1-Inputs!$E$70)+R75</f>
-        <v>9699.45213257267</v>
+        <v>9699.45213257268</v>
       </c>
       <c r="S89" s="51" t="n">
         <f aca="false">S74-S45*(1-Inputs!$E$70)+S75</f>
-        <v>9702.36879923933</v>
+        <v>9702.36879923935</v>
       </c>
       <c r="T89" s="51" t="n">
         <f aca="false">T74-T45*(1-Inputs!$E$70)+T75</f>
@@ -26314,19 +26314,19 @@
       </c>
       <c r="U89" s="51" t="n">
         <f aca="false">U74-U45*(1-Inputs!$E$70)+U75</f>
-        <v>9708.20213257267</v>
+        <v>9708.20213257268</v>
       </c>
       <c r="V89" s="51" t="n">
         <f aca="false">V74-V45*(1-Inputs!$E$70)+V75</f>
-        <v>9711.11879923934</v>
+        <v>9711.11879923935</v>
       </c>
       <c r="W89" s="51" t="n">
         <f aca="false">W74-W45*(1-Inputs!$E$70)+W75</f>
-        <v>9714.035465906</v>
+        <v>9714.03546590602</v>
       </c>
       <c r="X89" s="51" t="n">
         <f aca="false">X74-X45*(1-Inputs!$E$70)+X75</f>
-        <v>9716.95213257267</v>
+        <v>9716.95213257268</v>
       </c>
       <c r="Y89" s="51" t="n">
         <f aca="false">Y74-Y45*(1-Inputs!$E$70)+Y75</f>
@@ -26924,7 +26924,7 @@
       </c>
       <c r="AT93" s="51" t="n">
         <f aca="false">AS93+AT50</f>
-        <v>524338.862932106</v>
+        <v>524338.862932107</v>
       </c>
       <c r="AU93" s="51" t="n">
         <f aca="false">AT93+AU50</f>
@@ -27133,7 +27133,7 @@
       </c>
       <c r="AK94" s="58" t="n">
         <f aca="false">AK80+AK66+AK67+AK57</f>
-        <v>510466.32721347</v>
+        <v>510466.327213471</v>
       </c>
       <c r="AL94" s="58" t="n">
         <f aca="false">AL80+AL66+AL67+AL57</f>
@@ -27181,7 +27181,7 @@
       </c>
       <c r="AW94" s="58" t="n">
         <f aca="false">AW80+AW66+AW67+AW57</f>
-        <v>698296.439164199</v>
+        <v>698296.4391642</v>
       </c>
       <c r="AX94" s="58" t="n">
         <f aca="false">AX80+AX66+AX67+AX57</f>
@@ -27201,7 +27201,7 @@
       </c>
       <c r="BB94" s="58" t="n">
         <f aca="false">BB80+BB66+BB67+BB57</f>
-        <v>790210.948872361</v>
+        <v>790210.948872362</v>
       </c>
       <c r="BC94" s="58" t="n">
         <f aca="false">BC80+BC66+BC67+BC57</f>
@@ -27659,7 +27659,7 @@
       </c>
       <c r="AT96" s="51" t="n">
         <f aca="false">AT92+AT93</f>
-        <v>584338.862932106</v>
+        <v>584338.862932107</v>
       </c>
       <c r="AU96" s="51" t="n">
         <f aca="false">AU92+AU93</f>
@@ -27816,7 +27816,7 @@
       </c>
       <c r="X97" s="58" t="n">
         <f aca="false">X95+X96</f>
-        <v>332919.725232586</v>
+        <v>332919.725232587</v>
       </c>
       <c r="Y97" s="58" t="n">
         <f aca="false">Y95+Y96</f>
@@ -27844,7 +27844,7 @@
       </c>
       <c r="AE97" s="58" t="n">
         <f aca="false">AE95+AE96</f>
-        <v>429365.92851593</v>
+        <v>429365.928515931</v>
       </c>
       <c r="AF97" s="58" t="n">
         <f aca="false">AF95+AF96</f>
@@ -27860,7 +27860,7 @@
       </c>
       <c r="AI97" s="58" t="n">
         <f aca="false">AI95+AI96</f>
-        <v>471466.40832839</v>
+        <v>471466.408328391</v>
       </c>
       <c r="AJ97" s="58" t="n">
         <f aca="false">AJ95+AJ96</f>
@@ -27912,7 +27912,7 @@
       </c>
       <c r="AV97" s="58" t="n">
         <f aca="false">AV95+AV96</f>
-        <v>665908.333315047</v>
+        <v>665908.333315048</v>
       </c>
       <c r="AW97" s="58" t="n">
         <f aca="false">AW95+AW96</f>
@@ -27928,7 +27928,7 @@
       </c>
       <c r="AZ97" s="58" t="n">
         <f aca="false">AZ95+AZ96</f>
-        <v>757103.678383647</v>
+        <v>757103.678383648</v>
       </c>
       <c r="BA97" s="58" t="n">
         <f aca="false">BA95+BA96</f>
@@ -33004,7 +33004,7 @@
       </c>
       <c r="F18" s="35" t="n">
         <f aca="false">'P&amp;L'!F24</f>
-        <v>-65004.7628876924</v>
+        <v>-65004.7628876925</v>
       </c>
       <c r="H18" s="35" t="n">
         <f aca="false">INDEX(Monthly!$C$49:$BJ$49,($R$2-1)*12+1)</f>
@@ -35718,7 +35718,7 @@
       </c>
       <c r="B35" s="51" t="n">
         <f aca="false">IF($A35&gt;B$33,SUMPRODUCT($B$17:$F$17/(1+$A35)^$B$14:$F$14)+$F$17*(1+B$33)/($A35-B$33)/(1+$A35)^$F$14,"n/a")</f>
-        <v>1374481.18483667</v>
+        <v>1374481.18483666</v>
       </c>
       <c r="C35" s="51" t="n">
         <f aca="false">IF($A35&gt;C$33,SUMPRODUCT($B$17:$F$17/(1+$A35)^$B$14:$F$14)+$F$17*(1+C$33)/($A35-C$33)/(1+$A35)^$F$14,"n/a")</f>
@@ -36399,7 +36399,7 @@
       </c>
       <c r="C13" s="72" t="n">
         <f aca="false">IF(('Balance Sheet'!C12-'Balance Sheet'!C11)&lt;=0,"n/a",('Balance Sheet'!C5+'Balance Sheet'!C6+'Balance Sheet'!C7)/('Balance Sheet'!C12-'Balance Sheet'!C11))</f>
-        <v>9.62897283771879</v>
+        <v>9.6289728377188</v>
       </c>
       <c r="D13" s="72" t="n">
         <f aca="false">IF(('Balance Sheet'!D12-'Balance Sheet'!D11)&lt;=0,"n/a",('Balance Sheet'!D5+'Balance Sheet'!D6+'Balance Sheet'!D7)/('Balance Sheet'!D12-'Balance Sheet'!D11))</f>
@@ -36459,7 +36459,7 @@
       </c>
       <c r="E15" s="39" t="n">
         <f aca="false">IF('Balance Sheet'!E9&lt;=0,"n/a",'P&amp;L'!E25/'Balance Sheet'!E9)</f>
-        <v>0.281586318034303</v>
+        <v>0.281586318034302</v>
       </c>
       <c r="F15" s="39" t="n">
         <f aca="false">IF('Balance Sheet'!F9&lt;=0,"n/a",'P&amp;L'!F25/'Balance Sheet'!F9)</f>
@@ -36481,7 +36481,7 @@
       </c>
       <c r="D16" s="39" t="n">
         <f aca="false">IF('Balance Sheet'!D15&lt;=0,"n/a",'P&amp;L'!D25/'Balance Sheet'!D15)</f>
-        <v>0.361999900076399</v>
+        <v>0.361999900076398</v>
       </c>
       <c r="E16" s="39" t="n">
         <f aca="false">IF('Balance Sheet'!E15&lt;=0,"n/a",'P&amp;L'!E25/'Balance Sheet'!E15)</f>
@@ -36610,7 +36610,7 @@
       </c>
       <c r="D23" s="74" t="n">
         <f aca="false">IF(AND(ISNUMBER(D20),ISNUMBER(D21),ISNUMBER(D22)),D20*D21*D22,"n/a")</f>
-        <v>0.361999900076399</v>
+        <v>0.361999900076398</v>
       </c>
       <c r="E23" s="74" t="n">
         <f aca="false">IF(AND(ISNUMBER(E20),ISNUMBER(E21),ISNUMBER(E22)),E20*E21*E22,"n/a")</f>
@@ -39220,7 +39220,7 @@
       </c>
       <c r="F24" s="51" t="n">
         <f aca="false">SUMIF(Monthly!$C$5:$BJ$5,F$3,Monthly!$C$49:$BJ$49)</f>
-        <v>-65004.7628876924</v>
+        <v>-65004.7628876925</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>